<commit_message>
docs: update data dictionary with current Dataform definitions
</commit_message>
<xml_diff>
--- a/docs/polaris_v6_data_dictionary_v3.xlsx
+++ b/docs/polaris_v6_data_dictionary_v3.xlsx
@@ -20,6 +20,7 @@
     <sheet name="10_GitHub_Repo" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="11_Run_Registry" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="12_Forecast_Tool" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13_LCOE_Pipeline_Dataform" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -135,7 +136,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -235,6 +236,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -366,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -502,6 +508,20 @@
     <xf numFmtId="0" fontId="17" fillId="20" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -867,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1237,6 +1257,33 @@
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>13_LCOE_Pipeline_Dataform</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Dataform definitions: 12 .sqlx files, renames, dependency DAG, open flags</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>✅ Complete</t>
         </is>
@@ -2555,11 +2602,6 @@
           <t>Section 1 — Tables &amp; Views</t>
         </is>
       </c>
-      <c r="B4" s="42" t="n"/>
-      <c r="C4" s="42" t="n"/>
-      <c r="D4" s="42" t="n"/>
-      <c r="E4" s="42" t="n"/>
-      <c r="F4" s="42" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="43" t="inlineStr">
@@ -2759,11 +2801,6 @@
           <t>Section 2 — Run ID concept (TWO independent run_ids today)</t>
         </is>
       </c>
-      <c r="B12" s="42" t="n"/>
-      <c r="C12" s="42" t="n"/>
-      <c r="D12" s="42" t="n"/>
-      <c r="E12" s="42" t="n"/>
-      <c r="F12" s="42" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -2792,10 +2829,10 @@
           <t>Generated when the LCOE Model workbook (Case 4 / Case 7 / Case 8 / Budget) pushes via the consolidated Apps Script. Lives in polaris_raw.v6_raw_inputs_tab, v6_raw_capex_tool, v6_raw_opex_tool, etc. Feeds the full LCOE pipeline through to fct_finance.lcoe_facility_summary.</t>
         </is>
       </c>
-      <c r="C14" s="49" t="n"/>
-      <c r="D14" s="49" t="n"/>
-      <c r="E14" s="49" t="n"/>
-      <c r="F14" s="49" t="n"/>
+      <c r="C14" s="46" t="n"/>
+      <c r="D14" s="46" t="n"/>
+      <c r="E14" s="46" t="n"/>
+      <c r="F14" s="47" t="n"/>
     </row>
     <row r="15" ht="70" customHeight="1">
       <c r="A15" s="48" t="inlineStr">
@@ -2808,10 +2845,10 @@
           <t>Generated when the Forecast Tool workbook pushes via v6_forecast_ingest.gs. Lives in polaris_raw.v6_raw_forecast_inputs and the staging/aggregation objects in stg_finance. Does NOT flow into the LCOE fct layer today.</t>
         </is>
       </c>
-      <c r="C15" s="49" t="n"/>
-      <c r="D15" s="49" t="n"/>
-      <c r="E15" s="49" t="n"/>
-      <c r="F15" s="49" t="n"/>
+      <c r="C15" s="46" t="n"/>
+      <c r="D15" s="46" t="n"/>
+      <c r="E15" s="46" t="n"/>
+      <c r="F15" s="47" t="n"/>
     </row>
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="48" t="inlineStr">
@@ -2824,10 +2861,10 @@
           <t>NOT LINKED. The two run_ids are independent. A forecast push never updates the LCOE pipeline, and an LCOE push never updates the forecast tables.</t>
         </is>
       </c>
-      <c r="C16" s="49" t="n"/>
-      <c r="D16" s="49" t="n"/>
-      <c r="E16" s="49" t="n"/>
-      <c r="F16" s="49" t="n"/>
+      <c r="C16" s="46" t="n"/>
+      <c r="D16" s="46" t="n"/>
+      <c r="E16" s="46" t="n"/>
+      <c r="F16" s="47" t="n"/>
     </row>
     <row r="17" ht="70" customHeight="1">
       <c r="A17" s="48" t="inlineStr">
@@ -2840,10 +2877,10 @@
           <t>Always specify which run_id you are querying. Never join one set of tables to the other on run_id alone — the values come from independent ID sequences and a coincidental match would be meaningless. Linking is pending Dataform + automation work (FMA-118, FMA-60/85).</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n"/>
-      <c r="D17" s="49" t="n"/>
-      <c r="E17" s="49" t="n"/>
-      <c r="F17" s="49" t="n"/>
+      <c r="C17" s="46" t="n"/>
+      <c r="D17" s="46" t="n"/>
+      <c r="E17" s="46" t="n"/>
+      <c r="F17" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="41" t="inlineStr">
@@ -2851,11 +2888,6 @@
           <t>Section 3 — Export Log (lives in the Forecast Tool Google Sheet)</t>
         </is>
       </c>
-      <c r="B19" s="42" t="n"/>
-      <c r="C19" s="42" t="n"/>
-      <c r="D19" s="42" t="n"/>
-      <c r="E19" s="42" t="n"/>
-      <c r="F19" s="42" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="43" t="inlineStr">
@@ -2884,10 +2916,10 @@
           <t>Every successful push to BQ writes a single row to the 'Export Log' tab inside the Forecast Tool workbook. FP&amp;A users browse this tab to find the run_id they want without opening BigQuery.</t>
         </is>
       </c>
-      <c r="C21" s="49" t="n"/>
-      <c r="D21" s="49" t="n"/>
-      <c r="E21" s="49" t="n"/>
-      <c r="F21" s="49" t="n"/>
+      <c r="C21" s="46" t="n"/>
+      <c r="D21" s="46" t="n"/>
+      <c r="E21" s="46" t="n"/>
+      <c r="F21" s="47" t="n"/>
     </row>
     <row r="22" ht="55" customHeight="1">
       <c r="A22" s="48" t="inlineStr">
@@ -2900,10 +2932,10 @@
           <t>run_id · run_label · run_type · pushed_at · pushed_by · forecast_scenario_note · wind_rows · bess_rows · gas_rows · dtc_rows · solar_rows · total_rows</t>
         </is>
       </c>
-      <c r="C22" s="49" t="n"/>
-      <c r="D22" s="49" t="n"/>
-      <c r="E22" s="49" t="n"/>
-      <c r="F22" s="49" t="n"/>
+      <c r="C22" s="46" t="n"/>
+      <c r="D22" s="46" t="n"/>
+      <c r="E22" s="46" t="n"/>
+      <c r="F22" s="47" t="n"/>
     </row>
     <row r="23" ht="55" customHeight="1">
       <c r="A23" s="48" t="inlineStr">
@@ -2916,10 +2948,10 @@
           <t>Newest push at the TOP (row 2), older pushes below. Headers in row 1 are bold + frozen.</t>
         </is>
       </c>
-      <c r="C23" s="49" t="n"/>
-      <c r="D23" s="49" t="n"/>
-      <c r="E23" s="49" t="n"/>
-      <c r="F23" s="49" t="n"/>
+      <c r="C23" s="46" t="n"/>
+      <c r="D23" s="46" t="n"/>
+      <c r="E23" s="46" t="n"/>
+      <c r="F23" s="47" t="n"/>
     </row>
     <row r="24" ht="55" customHeight="1">
       <c r="A24" s="48" t="inlineStr">
@@ -2932,10 +2964,10 @@
           <t>Append-only. Existing log rows are never overwritten or deleted by the script. If the Export Log write fails for some reason, the BQ push still succeeds; a warning surfaces in the success modal.</t>
         </is>
       </c>
-      <c r="C24" s="49" t="n"/>
-      <c r="D24" s="49" t="n"/>
-      <c r="E24" s="49" t="n"/>
-      <c r="F24" s="49" t="n"/>
+      <c r="C24" s="46" t="n"/>
+      <c r="D24" s="46" t="n"/>
+      <c r="E24" s="46" t="n"/>
+      <c r="F24" s="47" t="n"/>
     </row>
     <row r="25" ht="55" customHeight="1">
       <c r="A25" s="48" t="inlineStr">
@@ -2948,10 +2980,10 @@
           <t>Adapted from Alexa's getOrCreateRunLog() in Polaris_GAS_Export.js. The forecast version differs from hers in tab name ('Export Log' vs 'Polaris Run Log') and ordering (newest-on-top vs append-bottom).</t>
         </is>
       </c>
-      <c r="C25" s="49" t="n"/>
-      <c r="D25" s="49" t="n"/>
-      <c r="E25" s="49" t="n"/>
-      <c r="F25" s="49" t="n"/>
+      <c r="C25" s="46" t="n"/>
+      <c r="D25" s="46" t="n"/>
+      <c r="E25" s="46" t="n"/>
+      <c r="F25" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
@@ -2959,11 +2991,6 @@
           <t>Section 4 — Modal window fields (mandatory before push)</t>
         </is>
       </c>
-      <c r="B27" s="42" t="n"/>
-      <c r="C27" s="42" t="n"/>
-      <c r="D27" s="42" t="n"/>
-      <c r="E27" s="42" t="n"/>
-      <c r="F27" s="42" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="43" t="inlineStr">
@@ -3010,8 +3037,8 @@
           <t>forecast_scenario_note (and run_notes for backward compat)</t>
         </is>
       </c>
-      <c r="E29" s="49" t="n"/>
-      <c r="F29" s="49" t="n"/>
+      <c r="E29" s="46" t="n"/>
+      <c r="F29" s="47" t="n"/>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="48" t="inlineStr">
@@ -3034,8 +3061,8 @@
           <t>run_label</t>
         </is>
       </c>
-      <c r="E30" s="49" t="n"/>
-      <c r="F30" s="49" t="n"/>
+      <c r="E30" s="46" t="n"/>
+      <c r="F30" s="47" t="n"/>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="48" t="inlineStr">
@@ -3058,8 +3085,8 @@
           <t>run_type</t>
         </is>
       </c>
-      <c r="E31" s="49" t="n"/>
-      <c r="F31" s="49" t="n"/>
+      <c r="E31" s="46" t="n"/>
+      <c r="F31" s="47" t="n"/>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="48" t="inlineStr">
@@ -3082,8 +3109,8 @@
           <t>solar_note</t>
         </is>
       </c>
-      <c r="E32" s="49" t="n"/>
-      <c r="F32" s="49" t="n"/>
+      <c r="E32" s="46" t="n"/>
+      <c r="F32" s="47" t="n"/>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="48" t="inlineStr">
@@ -3106,8 +3133,8 @@
           <t>wind_note</t>
         </is>
       </c>
-      <c r="E33" s="49" t="n"/>
-      <c r="F33" s="49" t="n"/>
+      <c r="E33" s="46" t="n"/>
+      <c r="F33" s="47" t="n"/>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="48" t="inlineStr">
@@ -3130,8 +3157,8 @@
           <t>bess_note</t>
         </is>
       </c>
-      <c r="E34" s="49" t="n"/>
-      <c r="F34" s="49" t="n"/>
+      <c r="E34" s="46" t="n"/>
+      <c r="F34" s="47" t="n"/>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="48" t="inlineStr">
@@ -3154,8 +3181,8 @@
           <t>gas_note</t>
         </is>
       </c>
-      <c r="E35" s="49" t="n"/>
-      <c r="F35" s="49" t="n"/>
+      <c r="E35" s="46" t="n"/>
+      <c r="F35" s="47" t="n"/>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="48" t="inlineStr">
@@ -3178,8 +3205,8 @@
           <t>dtc_note</t>
         </is>
       </c>
-      <c r="E36" s="49" t="n"/>
-      <c r="F36" s="49" t="n"/>
+      <c r="E36" s="46" t="n"/>
+      <c r="F36" s="47" t="n"/>
     </row>
     <row r="37" ht="75" customHeight="1">
       <c r="A37" s="48" t="inlineStr">
@@ -3192,10 +3219,10 @@
           <t>Project (hardcoded 'Roman III'), and per-tech: Last Actuals Date (Inputs (Tech)!AK4), Capacity + Units (Inputs_Capex!C11–C14), NTP (Construction Payments!E2/F2), COD (Construction Payments!E3/F3). Missing cells render as '—'. BESS / Gas / DTC have no NTP/COD/last-actuals cells in the workbook today; Gas has no capacity row either.</t>
         </is>
       </c>
-      <c r="C37" s="49" t="n"/>
-      <c r="D37" s="49" t="n"/>
-      <c r="E37" s="49" t="n"/>
-      <c r="F37" s="49" t="n"/>
+      <c r="C37" s="46" t="n"/>
+      <c r="D37" s="46" t="n"/>
+      <c r="E37" s="46" t="n"/>
+      <c r="F37" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="41" t="inlineStr">
@@ -3203,11 +3230,6 @@
           <t>Section 5 — Open questions / flags</t>
         </is>
       </c>
-      <c r="B39" s="42" t="n"/>
-      <c r="C39" s="42" t="n"/>
-      <c r="D39" s="42" t="n"/>
-      <c r="E39" s="42" t="n"/>
-      <c r="F39" s="42" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="43" t="inlineStr">
@@ -3263,7 +3285,7 @@
           <t>FMA-121</t>
         </is>
       </c>
-      <c r="F41" s="49" t="n"/>
+      <c r="F41" s="47" t="n"/>
     </row>
     <row r="42" ht="85" customHeight="1">
       <c r="A42" s="50" t="inlineStr">
@@ -3291,7 +3313,7 @@
           <t>FMA-113 (closed) — followup TBD</t>
         </is>
       </c>
-      <c r="F42" s="49" t="n"/>
+      <c r="F42" s="47" t="n"/>
     </row>
     <row r="43" ht="85" customHeight="1">
       <c r="A43" s="50" t="inlineStr">
@@ -3319,7 +3341,7 @@
           <t>FMA-118 (Dataform) · FMA-60 / FMA-85 (automation)</t>
         </is>
       </c>
-      <c r="F43" s="49" t="n"/>
+      <c r="F43" s="47" t="n"/>
     </row>
     <row r="44" ht="85" customHeight="1">
       <c r="A44" s="50" t="inlineStr">
@@ -3347,7 +3369,7 @@
           <t>FMA-108 / FMA-120 / FMA-121</t>
         </is>
       </c>
-      <c r="F44" s="49" t="n"/>
+      <c r="F44" s="47" t="n"/>
     </row>
     <row r="45" ht="85" customHeight="1">
       <c r="A45" s="50" t="inlineStr">
@@ -3375,7 +3397,7 @@
           <t>TBD — fix in source workbook or in staging</t>
         </is>
       </c>
-      <c r="F45" s="49" t="n"/>
+      <c r="F45" s="47" t="n"/>
     </row>
     <row r="46" ht="85" customHeight="1">
       <c r="A46" s="50" t="inlineStr">
@@ -3403,7 +3425,7 @@
           <t>FMA-118 (Dataform automation will resolve)</t>
         </is>
       </c>
-      <c r="F46" s="49" t="n"/>
+      <c r="F46" s="47" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="33">
@@ -3445,6 +3467,1487 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F66"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>LCOE Pipeline — Dataform Definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>Workspace: sandbox-lakehouse / us-south1 / lcoe-pipeline / test-lcoe-raw-data · As of 2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>Section 1 — 12 Dataform definitions (definitions/*.sqlx)</t>
+        </is>
+      </c>
+      <c r="B4" s="42" t="n"/>
+      <c r="C4" s="42" t="n"/>
+      <c r="D4" s="42" t="n"/>
+      <c r="E4" s="42" t="n"/>
+      <c r="F4" s="42" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="43" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C5" s="43" t="inlineStr">
+        <is>
+          <t>Target dataset</t>
+        </is>
+      </c>
+      <c r="D5" s="43" t="inlineStr">
+        <is>
+          <t>Output table</t>
+        </is>
+      </c>
+      <c r="E5" s="43" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F5" s="43" t="inlineStr">
+        <is>
+          <t>Key output columns / dependencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="105" customHeight="1">
+      <c r="A6" s="44" t="inlineStr">
+        <is>
+          <t>01_v6_master_staging.sqlx</t>
+        </is>
+      </c>
+      <c r="B6" s="45" t="inlineStr">
+        <is>
+          <t>operations
+(writes 12 tables)</t>
+        </is>
+      </c>
+      <c r="C6" s="44" t="inlineStr">
+        <is>
+          <t>stg_finance</t>
+        </is>
+      </c>
+      <c r="D6" s="44" t="inlineStr">
+        <is>
+          <t>v6_stg_lcoe_model_controls; v6_stg_project_timeline; v6_stg_project_capacity; v6_stg_generation_seasonality; v6_stg_degradation; v6_stg_tax_attributes; v6_stg_financing_fees; v6_stg_contingency; v6_stg_capex_unit_cost; v6_stg_opex_rates; v6_stg_insurance; v6_stg_property_tax</t>
+        </is>
+      </c>
+      <c r="E6" s="45" t="inlineStr">
+        <is>
+          <t>Master staging operation. Reads polaris_raw.v6_raw_inputs_tab + v6_raw_capex_tool and normalizes the raw long-format inputs into 12 domain-specific staging tables via CREATE OR REPLACE. NOT incremental — full overwrite on every run.</t>
+        </is>
+      </c>
+      <c r="F6" s="45" t="inlineStr">
+        <is>
+          <t>Each table keyed on (run_id, technology). Source row ranges documented in file header (LCOE Drivers R3-R10, Dates R13-R21, Capacities R23-R47, Tax R49-R97, Underwriting R99-R103, CAPEX R109-R152, OPEX R154-R215, Other Expenses R216-R336, Gas-Specific R338-R356, DTC-Specific R358-R368).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="105" customHeight="1">
+      <c r="A7" s="44" t="inlineStr">
+        <is>
+          <t>02_v6_silver_consolidated.sqlx</t>
+        </is>
+      </c>
+      <c r="B7" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="inlineStr">
+        <is>
+          <t>mart_finance</t>
+        </is>
+      </c>
+      <c r="D7" s="44" t="inlineStr">
+        <is>
+          <t>v6_silver_itc_inputs</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="inlineStr">
+        <is>
+          <t>Computes ITC, depreciable basis, and MACRS basis dollar amounts. Joins stg_tax_attributes + stg_capex_unit_cost + stg_financing_fees + stg_project_timeline. INCREMENTAL — new run_ids appended; existing skipped.</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>gross_itc_usd; net_itc_usd; depreciable_basis_usd; five_yr_macrs_basis_usd; twenty_yr_macrs_basis_usd; bonus_dep_switch; ptc_* (placeholder fields); placed_in_service_date; substantial_completion_date; underwriting_fee_usd; transfer_transaction_cost_usd · Depends on: 01_v6_master_staging</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="105" customHeight="1">
+      <c r="A8" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_project_timeline_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="B8" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="inlineStr">
+        <is>
+          <t>project_timeline_monthly</t>
+        </is>
+      </c>
+      <c r="E8" s="45" t="inlineStr">
+        <is>
+          <t>CROSS JOIN dim_time.dim_month × 5 techs. Computes is_development, is_construction, is_operation phase flags + operating_year_num/operating_month_num. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>calendar_month_end; technology; is_development; is_construction; is_operation; operating_year_num; operating_month_num; run_id; pushed_at · Depends on: 01_v6_master_staging (uses stg_project_timeline + dim_time.dim_month)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_generation_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="B9" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>generation_monthly</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="inlineStr">
+        <is>
+          <t>Monthly generation (MWh) for Solar/Wind/Gas. y1_monthly_gen × degradation_factor. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F9" s="45" t="inlineStr">
+        <is>
+          <t>calendar_month_end; technology; generation_mwh; operating_year_num; run_id; pushed_at · Depends on: project_timeline_monthly + mart_finance.v6_silver_project_inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="105" customHeight="1">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_project_capex_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="B10" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>project_capex_monthly</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="inlineStr">
+        <is>
+          <t>UNPIVOT 577 period_* columns from v6_raw_capex_tool. Deduplicates duplicate per-tech blocks via ROW_NUMBER(). SAFE_CAST handles 2 STRING-typed period cols. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>calendar_month_end; technology; monthly_capex_usd; component_count; run_id; pushed_at · Depends on: 01_v6_master_staging (reads raw capex tool directly)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="105" customHeight="1">
+      <c r="A11" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_revenue_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="B11" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>revenue_monthly</t>
+        </is>
+      </c>
+      <c r="E11" s="45" t="inlineStr">
+        <is>
+          <t>$0 PLACEHOLDER. OI-005: market curves pending Brian Wile. Every operating month gets is_placeholder=TRUE and revenue_usd=0. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F11" s="45" t="inlineStr">
+        <is>
+          <t>calendar_month_end; technology; revenue_usd (0); is_placeholder (TRUE); placeholder_reason; run_id; pushed_at · Depends on: project_timeline_monthly</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="105" customHeight="1">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_tax_credit_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="B12" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D12" s="44" t="inlineStr">
+        <is>
+          <t>tax_credit_monthly</t>
+        </is>
+      </c>
+      <c r="E12" s="45" t="inlineStr">
+        <is>
+          <t>ITC posted as a single negative lump on the month of substantial completion. PTC zero until OI-005 resolved. Sign convention: stored negative so + total_itc_usd subtracts from LCOE numerator. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F12" s="45" t="inlineStr">
+        <is>
+          <t>calendar_month_end; technology; itc_usd (negative); ptc_usd (0); run_id; pushed_at · Depends on: project_timeline_monthly + v6_silver_itc_inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="105" customHeight="1">
+      <c r="A13" s="51" t="inlineStr">
+        <is>
+          <t>04_v6_stg_opex_lifetime_totals.sqlx</t>
+        </is>
+      </c>
+      <c r="B13" s="52" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C13" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance ⚠</t>
+        </is>
+      </c>
+      <c r="D13" s="51" t="inlineStr">
+        <is>
+          <t>stg_opex_lifetime_totals</t>
+        </is>
+      </c>
+      <c r="E13" s="52" t="inlineStr">
+        <is>
+          <t>Pre-aggregates per-tech lifetime opex totals from v6_raw_opex_tool. File name says 'stg' but writes to fct_finance — see Section 2 renames. Used as the opex source for project_opex_monthly and lcoe_facility_summary. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F13" s="52" t="inlineStr">
+        <is>
+          <t>technology; om_lifetime_usd; land_lease_lifetime_usd; insurance_lifetime_usd; property_tax_lifetime_usd; other_exp_lifetime_usd; franchise_tax_lifetime_usd; sleeve_fee_lifetime_usd; gas_fuel_lifetime_usd; dtc_hv_lifetime_usd; wake_losses_lifetime_usd; operating_lcs_lifetime_usd; run_id; pushed_at · Depends on: project_timeline_monthly</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="105" customHeight="1">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>05_project_opex_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D14" s="44" t="inlineStr">
+        <is>
+          <t>project_opex_monthly</t>
+        </is>
+      </c>
+      <c r="E14" s="45" t="inlineStr">
+        <is>
+          <t>Monthly opex per tech, 12 components. Optimized: computes annual then divides by 12 to reduce join fan-out. LCs kept at monthly grain due to date-range logic. INCREMENTAL. Known gaps: OI-009 BESS/DTC Covered O&amp;M = 0.</t>
+        </is>
+      </c>
+      <c r="F14" s="45" t="inlineStr">
+        <is>
+          <t>om_monthly_usd; land_lease_monthly_usd; insurance_monthly_usd; property_tax_monthly_usd; other_expenses_monthly_usd; franchise_tax_monthly_usd; sleeve_fee_monthly_usd; gas_fuel_monthly_usd; dtc_hv_monthly_usd; lcs_monthly_usd; wake_losses_monthly_usd; total_opex_monthly_usd; has_missing_om_inputs · Depends on: stg_opex_lifetime_totals + project_timeline_monthly + stg_finance.v6_stg_operating_lcs (legacy, not in Dataform)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="105" customHeight="1">
+      <c r="A15" s="44" t="inlineStr">
+        <is>
+          <t>07_v6_fct_depreciation_monthly_1.sqlx</t>
+        </is>
+      </c>
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C15" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D15" s="44" t="inlineStr">
+        <is>
+          <t>depreciation_monthly</t>
+        </is>
+      </c>
+      <c r="E15" s="45" t="inlineStr">
+        <is>
+          <t>MACRS depreciation tax shield monthly. Annual = basis × depreciation_pct × effective_tax_rate. Monthly = annual ÷ 12. Year 21 half-year handled as full year on last month. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F15" s="45" t="inlineStr">
+        <is>
+          <t>calendar_month_end; technology; dep_shield_monthly_usd; operating_year_num; run_id; pushed_at · Depends on: project_opex_monthly + project_timeline_monthly + v6_silver_itc_inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="105" customHeight="1">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>08_v6_fct_lcoe_component_annual.sqlx</t>
+        </is>
+      </c>
+      <c r="B16" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D16" s="44" t="inlineStr">
+        <is>
+          <t>lcoe_component_annual</t>
+        </is>
+      </c>
+      <c r="E16" s="45" t="inlineStr">
+        <is>
+          <t>Per-tech annual LCOE numerator/denominator. Solar/Wind/Gas/BESS/DTC. Solar/Wind opex capped at DTC end of life (2049-03-31, commented filter). BESS/Gas denominators hardcoded 1150/1200 MW — TODO pull from silver_capex.</t>
+        </is>
+      </c>
+      <c r="F16" s="45" t="inlineStr">
+        <is>
+          <t>technology; lcoe_usd_per_unit; lcoe_numerator_usd; lcoe_denominator; lcoe_denominator_unit; total_capex_usd; total_opex_usd; total_itc_usd; total_dep_shield_usd; total_revenue_usd · Depends on: depreciation_monthly, project_capex_monthly, project_opex_monthly, tax_credit_monthly, generation_monthly, revenue_monthly, project_timeline_monthly</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="105" customHeight="1">
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>09_v6_fct_lcoe_facility_summary.sqlx</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="inlineStr">
+        <is>
+          <t>incremental</t>
+        </is>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
+        <is>
+          <t>fct_finance</t>
+        </is>
+      </c>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>lcoe_facility_summary</t>
+        </is>
+      </c>
+      <c r="E17" s="45" t="inlineStr">
+        <is>
+          <t>Final LCOE numbers per tech + a 'Facility' total row. Facility denominator HARDCODED 175,200,000 MWh (DTC consumption). Facility opex sourced from stg_opex_lifetime_totals (includes pre-SC months). DTC excluded from Facility numerator per workbook design. INCREMENTAL.</t>
+        </is>
+      </c>
+      <c r="F17" s="45" t="inlineStr">
+        <is>
+          <t>technology (5 techs + 'Facility'); lcoe_usd_per_unit; lcoe_denominator_unit; total_capex_usd; total_opex_usd; total_itc_usd; total_dep_shield_usd; total_revenue_usd; lcoe_numerator_usd; lcoe_denominator · Depends on: lcoe_component_annual + stg_opex_lifetime_totals</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>Section 2 — Renamed / moved objects (Dataform vs manual SQL)</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="n"/>
+      <c r="C19" s="42" t="n"/>
+      <c r="D19" s="42" t="n"/>
+      <c r="E19" s="42" t="n"/>
+      <c r="F19" s="42" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="43" t="inlineStr">
+        <is>
+          <t>Old (legacy / still in BQ)</t>
+        </is>
+      </c>
+      <c r="B20" s="43" t="inlineStr">
+        <is>
+          <t>New (Dataform output)</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
+        <is>
+          <t>Change type</t>
+        </is>
+      </c>
+      <c r="D20" s="43" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E20" s="46" t="n"/>
+      <c r="F20" s="47" t="n"/>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_generation_monthly</t>
+        </is>
+      </c>
+      <c r="B21" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.generation_monthly</t>
+        </is>
+      </c>
+      <c r="C21" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D21" s="52" t="inlineStr">
+        <is>
+          <t>Both tables exist. Old last push 2026-06-21, new last push 2026-06-24.</t>
+        </is>
+      </c>
+      <c r="E21" s="53" t="n"/>
+      <c r="F21" s="53" t="n"/>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_project_capex_monthly</t>
+        </is>
+      </c>
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.project_capex_monthly</t>
+        </is>
+      </c>
+      <c r="C22" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D22" s="52" t="inlineStr">
+        <is>
+          <t>236 rows old, 9,901 rows new. Dataform is current.</t>
+        </is>
+      </c>
+      <c r="E22" s="53" t="n"/>
+      <c r="F22" s="53" t="n"/>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_project_timeline_monthly</t>
+        </is>
+      </c>
+      <c r="B23" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.project_timeline_monthly</t>
+        </is>
+      </c>
+      <c r="C23" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D23" s="52" t="inlineStr">
+        <is>
+          <t>Both populated; Dataform is the authoritative source going forward.</t>
+        </is>
+      </c>
+      <c r="E23" s="53" t="n"/>
+      <c r="F23" s="53" t="n"/>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_revenue_monthly</t>
+        </is>
+      </c>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.revenue_monthly</t>
+        </is>
+      </c>
+      <c r="C24" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D24" s="52" t="inlineStr">
+        <is>
+          <t>$0 placeholder either way.</t>
+        </is>
+      </c>
+      <c r="E24" s="53" t="n"/>
+      <c r="F24" s="53" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_tax_credit_monthly</t>
+        </is>
+      </c>
+      <c r="B25" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.tax_credit_monthly</t>
+        </is>
+      </c>
+      <c r="C25" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D25" s="52" t="inlineStr"/>
+      <c r="E25" s="53" t="n"/>
+      <c r="F25" s="53" t="n"/>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_project_opex_monthly</t>
+        </is>
+      </c>
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.project_opex_monthly</t>
+        </is>
+      </c>
+      <c r="C26" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D26" s="52" t="inlineStr">
+        <is>
+          <t>1,500 rows old, 77,999 rows new. Dataform is current.</t>
+        </is>
+      </c>
+      <c r="E26" s="53" t="n"/>
+      <c r="F26" s="53" t="n"/>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_depreciation_monthly</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.depreciation_monthly</t>
+        </is>
+      </c>
+      <c r="C27" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D27" s="52" t="inlineStr"/>
+      <c r="E27" s="53" t="n"/>
+      <c r="F27" s="53" t="n"/>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_lcoe_component_annual</t>
+        </is>
+      </c>
+      <c r="B28" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.lcoe_component_annual</t>
+        </is>
+      </c>
+      <c r="C28" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D28" s="52" t="inlineStr"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="53" t="n"/>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.v6_fct_lcoe_facility_summary</t>
+        </is>
+      </c>
+      <c r="B29" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.lcoe_facility_summary</t>
+        </is>
+      </c>
+      <c r="C29" s="52" t="inlineStr">
+        <is>
+          <t>name (dropped v6_fct_ prefix)</t>
+        </is>
+      </c>
+      <c r="D29" s="52" t="inlineStr">
+        <is>
+          <t>6 rows old, 42 rows new.</t>
+        </is>
+      </c>
+      <c r="E29" s="53" t="n"/>
+      <c r="F29" s="53" t="n"/>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="51" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_opex_lifetime_totals</t>
+        </is>
+      </c>
+      <c r="B30" s="51" t="inlineStr">
+        <is>
+          <t>fct_finance.stg_opex_lifetime_totals</t>
+        </is>
+      </c>
+      <c r="C30" s="52" t="inlineStr">
+        <is>
+          <t>DATASET MOVE + name change</t>
+        </is>
+      </c>
+      <c r="D30" s="52" t="inlineStr">
+        <is>
+          <t>Moved from stg_finance to fct_finance and lost the v6_ prefix. Old last push 2026-06-15, new last push 2026-06-24.</t>
+        </is>
+      </c>
+      <c r="E30" s="53" t="n"/>
+      <c r="F30" s="53" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>Section 3 — Staging tables NOT created by Dataform (still need manual SQL)</t>
+        </is>
+      </c>
+      <c r="B32" s="42" t="n"/>
+      <c r="C32" s="42" t="n"/>
+      <c r="D32" s="42" t="n"/>
+      <c r="E32" s="42" t="n"/>
+      <c r="F32" s="42" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="43" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="B33" s="43" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C33" s="43" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D33" s="43" t="inlineStr">
+        <is>
+          <t>Used by</t>
+        </is>
+      </c>
+      <c r="E33" s="46" t="n"/>
+      <c r="F33" s="47" t="n"/>
+    </row>
+    <row r="34" ht="50" customHeight="1">
+      <c r="A34" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_franchise_tax</t>
+        </is>
+      </c>
+      <c r="B34" s="55" t="inlineStr">
+        <is>
+          <t>still in BQ</t>
+        </is>
+      </c>
+      <c r="C34" s="55" t="inlineStr">
+        <is>
+          <t>Franchise tax % of revenue per tech. Source: Inputs OpEx section.</t>
+        </is>
+      </c>
+      <c r="D34" s="55" t="inlineStr">
+        <is>
+          <t>Legacy v6_fct_* opex monthly path (deprecated).</t>
+        </is>
+      </c>
+      <c r="E34" s="56" t="n"/>
+      <c r="F34" s="56" t="n"/>
+    </row>
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_land_lease</t>
+        </is>
+      </c>
+      <c r="B35" s="55" t="inlineStr">
+        <is>
+          <t>still in BQ</t>
+        </is>
+      </c>
+      <c r="C35" s="55" t="inlineStr">
+        <is>
+          <t>Land lease toggle, $/acre, total acres, escalator. Source: Inputs OpEx.</t>
+        </is>
+      </c>
+      <c r="D35" s="55" t="inlineStr">
+        <is>
+          <t>Legacy path. Dataform uses stg_opex_lifetime_totals instead.</t>
+        </is>
+      </c>
+      <c r="E35" s="56" t="n"/>
+      <c r="F35" s="56" t="n"/>
+    </row>
+    <row r="36" ht="50" customHeight="1">
+      <c r="A36" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_other_expenses</t>
+        </is>
+      </c>
+      <c r="B36" s="55" t="inlineStr">
+        <is>
+          <t>still in BQ</t>
+        </is>
+      </c>
+      <c r="C36" s="55" t="inlineStr">
+        <is>
+          <t>21 named expense line items per tech (unit-aware). Source: Inputs Other Expenses R216-R336.</t>
+        </is>
+      </c>
+      <c r="D36" s="55" t="inlineStr">
+        <is>
+          <t>Legacy path.</t>
+        </is>
+      </c>
+      <c r="E36" s="56" t="n"/>
+      <c r="F36" s="56" t="n"/>
+    </row>
+    <row r="37" ht="50" customHeight="1">
+      <c r="A37" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_gas_opex</t>
+        </is>
+      </c>
+      <c r="B37" s="55" t="inlineStr">
+        <is>
+          <t>still in BQ</t>
+        </is>
+      </c>
+      <c r="C37" s="55" t="inlineStr">
+        <is>
+          <t>Heat rate, fuel price, FT volumes &amp; escalators. Source: Inputs Gas-Specific R338-R356.</t>
+        </is>
+      </c>
+      <c r="D37" s="55" t="inlineStr">
+        <is>
+          <t>Legacy path.</t>
+        </is>
+      </c>
+      <c r="E37" s="56" t="n"/>
+      <c r="F37" s="56" t="n"/>
+    </row>
+    <row r="38" ht="50" customHeight="1">
+      <c r="A38" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_dtc_opex</t>
+        </is>
+      </c>
+      <c r="B38" s="55" t="inlineStr">
+        <is>
+          <t>still in BQ</t>
+        </is>
+      </c>
+      <c r="C38" s="55" t="inlineStr">
+        <is>
+          <t>HV maintenance and insurance yr1 rates + escalators. Source: Inputs DTC-Specific R358-R368.</t>
+        </is>
+      </c>
+      <c r="D38" s="55" t="inlineStr">
+        <is>
+          <t>Legacy path.</t>
+        </is>
+      </c>
+      <c r="E38" s="56" t="n"/>
+      <c r="F38" s="56" t="n"/>
+    </row>
+    <row r="39" ht="50" customHeight="1">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_operating_lcs</t>
+        </is>
+      </c>
+      <c r="B39" s="55" t="inlineStr">
+        <is>
+          <t>still in BQ</t>
+        </is>
+      </c>
+      <c r="C39" s="55" t="inlineStr">
+        <is>
+          <t>LC label, start/end period, annual amount, escalation. One row per LC per tech.</t>
+        </is>
+      </c>
+      <c r="D39" s="55" t="inlineStr">
+        <is>
+          <t>ACTIVE — referenced by 05_project_opex_monthly.sqlx for the lcs_monthly_usd column. Dataform depends on this but does not create it.</t>
+        </is>
+      </c>
+      <c r="E39" s="56" t="n"/>
+      <c r="F39" s="56" t="n"/>
+    </row>
+    <row r="40" ht="50" customHeight="1">
+      <c r="A40" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_om_schedules</t>
+        </is>
+      </c>
+      <c r="B40" s="55" t="inlineStr">
+        <is>
+          <t>still in BQ</t>
+        </is>
+      </c>
+      <c r="C40" s="55" t="inlineStr">
+        <is>
+          <t>Monthly O&amp;M schedules per tech.</t>
+        </is>
+      </c>
+      <c r="D40" s="55" t="inlineStr">
+        <is>
+          <t>Possibly used by older opex calculation paths. Not in Dataform.</t>
+        </is>
+      </c>
+      <c r="E40" s="56" t="n"/>
+      <c r="F40" s="56" t="n"/>
+    </row>
+    <row r="41" ht="50" customHeight="1">
+      <c r="A41" s="54" t="inlineStr">
+        <is>
+          <t>stg_finance.v6_stg_opex_lifetime_totals</t>
+        </is>
+      </c>
+      <c r="B41" s="55" t="inlineStr">
+        <is>
+          <t>DUPLICATE</t>
+        </is>
+      </c>
+      <c r="C41" s="55" t="inlineStr">
+        <is>
+          <t>Old version in stg_finance still exists (last push 2026-06-15). Dataform now writes to fct_finance.stg_opex_lifetime_totals instead.</t>
+        </is>
+      </c>
+      <c r="D41" s="55" t="inlineStr">
+        <is>
+          <t>Stale. Should be retired.</t>
+        </is>
+      </c>
+      <c r="E41" s="56" t="n"/>
+      <c r="F41" s="56" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>Section 4 — Dependency order (Dataform DAG)</t>
+        </is>
+      </c>
+      <c r="B43" s="42" t="n"/>
+      <c r="C43" s="42" t="n"/>
+      <c r="D43" s="42" t="n"/>
+      <c r="E43" s="42" t="n"/>
+      <c r="F43" s="42" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="43" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B44" s="43" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="C44" s="43" t="inlineStr">
+        <is>
+          <t>Depends on</t>
+        </is>
+      </c>
+      <c r="D44" s="46" t="n"/>
+      <c r="E44" s="46" t="n"/>
+      <c r="F44" s="47" t="n"/>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>01_v6_master_staging.sqlx</t>
+        </is>
+      </c>
+      <c r="C45" s="45" t="inlineStr">
+        <is>
+          <t>(none — reads raw)</t>
+        </is>
+      </c>
+      <c r="D45" s="49" t="n"/>
+      <c r="E45" s="49" t="n"/>
+      <c r="F45" s="49" t="n"/>
+    </row>
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="48" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>02_v6_silver_consolidated.sqlx</t>
+        </is>
+      </c>
+      <c r="C46" s="45" t="inlineStr">
+        <is>
+          <t>01_v6_master_staging</t>
+        </is>
+      </c>
+      <c r="D46" s="49" t="n"/>
+      <c r="E46" s="49" t="n"/>
+      <c r="F46" s="49" t="n"/>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="48" t="inlineStr">
+        <is>
+          <t>3a</t>
+        </is>
+      </c>
+      <c r="B47" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_project_timeline_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="C47" s="45" t="inlineStr">
+        <is>
+          <t>01_v6_master_staging</t>
+        </is>
+      </c>
+      <c r="D47" s="49" t="n"/>
+      <c r="E47" s="49" t="n"/>
+      <c r="F47" s="49" t="n"/>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="48" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_project_capex_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="C48" s="45" t="inlineStr">
+        <is>
+          <t>01_v6_master_staging</t>
+        </is>
+      </c>
+      <c r="D48" s="49" t="n"/>
+      <c r="E48" s="49" t="n"/>
+      <c r="F48" s="49" t="n"/>
+    </row>
+    <row r="49" ht="24" customHeight="1">
+      <c r="A49" s="48" t="inlineStr">
+        <is>
+          <t>3c</t>
+        </is>
+      </c>
+      <c r="B49" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_generation_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="C49" s="45" t="inlineStr">
+        <is>
+          <t>project_timeline_monthly + v6_silver_project_inputs</t>
+        </is>
+      </c>
+      <c r="D49" s="49" t="n"/>
+      <c r="E49" s="49" t="n"/>
+      <c r="F49" s="49" t="n"/>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="A50" s="48" t="inlineStr">
+        <is>
+          <t>3d</t>
+        </is>
+      </c>
+      <c r="B50" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_revenue_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="C50" s="45" t="inlineStr">
+        <is>
+          <t>project_timeline_monthly</t>
+        </is>
+      </c>
+      <c r="D50" s="49" t="n"/>
+      <c r="E50" s="49" t="n"/>
+      <c r="F50" s="49" t="n"/>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="48" t="inlineStr">
+        <is>
+          <t>3e</t>
+        </is>
+      </c>
+      <c r="B51" s="44" t="inlineStr">
+        <is>
+          <t>03_v6_fct_tax_credit_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="C51" s="45" t="inlineStr">
+        <is>
+          <t>project_timeline_monthly + v6_silver_itc_inputs</t>
+        </is>
+      </c>
+      <c r="D51" s="49" t="n"/>
+      <c r="E51" s="49" t="n"/>
+      <c r="F51" s="49" t="n"/>
+    </row>
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="48" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="44" t="inlineStr">
+        <is>
+          <t>04_v6_stg_opex_lifetime_totals.sqlx</t>
+        </is>
+      </c>
+      <c r="C52" s="45" t="inlineStr">
+        <is>
+          <t>project_timeline_monthly</t>
+        </is>
+      </c>
+      <c r="D52" s="49" t="n"/>
+      <c r="E52" s="49" t="n"/>
+      <c r="F52" s="49" t="n"/>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="44" t="inlineStr">
+        <is>
+          <t>05_project_opex_monthly.sqlx</t>
+        </is>
+      </c>
+      <c r="C53" s="45" t="inlineStr">
+        <is>
+          <t>stg_opex_lifetime_totals + project_timeline_monthly + v6_stg_operating_lcs (legacy)</t>
+        </is>
+      </c>
+      <c r="D53" s="49" t="n"/>
+      <c r="E53" s="49" t="n"/>
+      <c r="F53" s="49" t="n"/>
+    </row>
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="48" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B54" s="44" t="inlineStr">
+        <is>
+          <t>07_v6_fct_depreciation_monthly_1.sqlx</t>
+        </is>
+      </c>
+      <c r="C54" s="45" t="inlineStr">
+        <is>
+          <t>project_opex_monthly + project_timeline_monthly + v6_silver_itc_inputs</t>
+        </is>
+      </c>
+      <c r="D54" s="49" t="n"/>
+      <c r="E54" s="49" t="n"/>
+      <c r="F54" s="49" t="n"/>
+    </row>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="48" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B55" s="44" t="inlineStr">
+        <is>
+          <t>08_v6_fct_lcoe_component_annual.sqlx</t>
+        </is>
+      </c>
+      <c r="C55" s="45" t="inlineStr">
+        <is>
+          <t>all step 3 + 5 + 7 + 4</t>
+        </is>
+      </c>
+      <c r="D55" s="49" t="n"/>
+      <c r="E55" s="49" t="n"/>
+      <c r="F55" s="49" t="n"/>
+    </row>
+    <row r="56" ht="24" customHeight="1">
+      <c r="A56" s="48" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B56" s="44" t="inlineStr">
+        <is>
+          <t>09_v6_fct_lcoe_facility_summary.sqlx</t>
+        </is>
+      </c>
+      <c r="C56" s="45" t="inlineStr">
+        <is>
+          <t>lcoe_component_annual + stg_opex_lifetime_totals</t>
+        </is>
+      </c>
+      <c r="D56" s="49" t="n"/>
+      <c r="E56" s="49" t="n"/>
+      <c r="F56" s="49" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="41" t="inlineStr">
+        <is>
+          <t>Section 5 — Open flags</t>
+        </is>
+      </c>
+      <c r="B58" s="42" t="n"/>
+      <c r="C58" s="42" t="n"/>
+      <c r="D58" s="42" t="n"/>
+      <c r="E58" s="42" t="n"/>
+      <c r="F58" s="42" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="43" t="inlineStr">
+        <is>
+          <t>Flag</t>
+        </is>
+      </c>
+      <c r="B59" s="43" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C59" s="43" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D59" s="43" t="inlineStr">
+        <is>
+          <t>Linked tickets</t>
+        </is>
+      </c>
+      <c r="E59" s="43" t="inlineStr"/>
+      <c r="F59" s="47" t="n"/>
+    </row>
+    <row r="60" ht="64" customHeight="1">
+      <c r="A60" s="50" t="inlineStr">
+        <is>
+          <t>BESS/Gas denominator hardcoded</t>
+        </is>
+      </c>
+      <c r="B60" s="45" t="inlineStr">
+        <is>
+          <t>lcoe_component_annual hardcodes BESS=1150 MW, Gas=1200 MW denominators. TODO in file: pull from silver_capex instead.</t>
+        </is>
+      </c>
+      <c r="C60" s="45" t="inlineStr">
+        <is>
+          <t>Arlind</t>
+        </is>
+      </c>
+      <c r="D60" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="49" t="n"/>
+      <c r="F60" s="49" t="n"/>
+    </row>
+    <row r="61" ht="64" customHeight="1">
+      <c r="A61" s="50" t="inlineStr">
+        <is>
+          <t>Facility denominator hardcoded</t>
+        </is>
+      </c>
+      <c r="B61" s="45" t="inlineStr">
+        <is>
+          <t>lcoe_facility_summary uses 175,200,000 MWh literal. Tied to DTC consumption assumption.</t>
+        </is>
+      </c>
+      <c r="C61" s="45" t="inlineStr">
+        <is>
+          <t>Alexa / Jim D</t>
+        </is>
+      </c>
+      <c r="D61" s="44" t="inlineStr">
+        <is>
+          <t>OI-008 / KI-008</t>
+        </is>
+      </c>
+      <c r="E61" s="49" t="n"/>
+      <c r="F61" s="49" t="n"/>
+    </row>
+    <row r="62" ht="64" customHeight="1">
+      <c r="A62" s="50" t="inlineStr">
+        <is>
+          <t>Revenue = $0 placeholder</t>
+        </is>
+      </c>
+      <c r="B62" s="45" t="inlineStr">
+        <is>
+          <t>03_v6_fct_revenue_monthly emits $0 for every operating month, flagged is_placeholder=TRUE.</t>
+        </is>
+      </c>
+      <c r="C62" s="45" t="inlineStr">
+        <is>
+          <t>Brian Wile</t>
+        </is>
+      </c>
+      <c r="D62" s="44" t="inlineStr">
+        <is>
+          <t>OI-005</t>
+        </is>
+      </c>
+      <c r="E62" s="49" t="n"/>
+      <c r="F62" s="49" t="n"/>
+    </row>
+    <row r="63" ht="64" customHeight="1">
+      <c r="A63" s="50" t="inlineStr">
+        <is>
+          <t>BESS/DTC O&amp;M missing</t>
+        </is>
+      </c>
+      <c r="B63" s="45" t="inlineStr">
+        <is>
+          <t>05_project_opex_monthly sets has_missing_om_inputs=TRUE when om_annual_usd=0 for BESS/DTC.</t>
+        </is>
+      </c>
+      <c r="C63" s="45" t="inlineStr">
+        <is>
+          <t>Brad Platt / Ted Mongan</t>
+        </is>
+      </c>
+      <c r="D63" s="44" t="inlineStr">
+        <is>
+          <t>OI-009</t>
+        </is>
+      </c>
+      <c r="E63" s="49" t="n"/>
+      <c r="F63" s="49" t="n"/>
+    </row>
+    <row r="64" ht="64" customHeight="1">
+      <c r="A64" s="50" t="inlineStr">
+        <is>
+          <t>v6_fct_* tables not cleaned up</t>
+        </is>
+      </c>
+      <c r="B64" s="45" t="inlineStr">
+        <is>
+          <t>9 legacy v6_fct_* tables and 1 legacy v6_stg_opex_lifetime_totals still exist in BQ with stale data (last push 2026-06-21 / -06-15). Should be dropped once downstream consumers point at the Dataform outputs.</t>
+        </is>
+      </c>
+      <c r="C64" s="45" t="inlineStr">
+        <is>
+          <t>Arlind</t>
+        </is>
+      </c>
+      <c r="D64" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="49" t="n"/>
+      <c r="F64" s="49" t="n"/>
+    </row>
+    <row r="65" ht="64" customHeight="1">
+      <c r="A65" s="50" t="inlineStr">
+        <is>
+          <t>6 staging tables not in Dataform</t>
+        </is>
+      </c>
+      <c r="B65" s="45" t="inlineStr">
+        <is>
+          <t>v6_stg_franchise_tax, v6_stg_land_lease, v6_stg_other_expenses, v6_stg_gas_opex, v6_stg_dtc_opex, v6_stg_operating_lcs, v6_stg_om_schedules still maintained via manual SQL. v6_stg_operating_lcs is actively referenced by 05_project_opex_monthly so it MUST keep being refreshed until migrated.</t>
+        </is>
+      </c>
+      <c r="C65" s="45" t="inlineStr">
+        <is>
+          <t>Alexa</t>
+        </is>
+      </c>
+      <c r="D65" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="49" t="n"/>
+      <c r="F65" s="49" t="n"/>
+    </row>
+    <row r="66" ht="64" customHeight="1">
+      <c r="A66" s="50" t="inlineStr">
+        <is>
+          <t>Solar 13.50 Owner construction case bug (unchanged)</t>
+        </is>
+      </c>
+      <c r="B66" s="45" t="inlineStr">
+        <is>
+          <t>Source workbook has 'Owner Construction' and 'Owner construction' as separate values for acct_code 13.50. Affects forecast tool only.</t>
+        </is>
+      </c>
+      <c r="C66" s="45" t="inlineStr">
+        <is>
+          <t>Source workbook</t>
+        </is>
+      </c>
+      <c r="D66" s="44" t="inlineStr">
+        <is>
+          <t>FMA-121</t>
+        </is>
+      </c>
+      <c r="E66" s="49" t="n"/>
+      <c r="F66" s="49" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="46">
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="D37:F37"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="D64:F64"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="C47:F47"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="C44:F44"/>
+    <mergeCell ref="D63:F63"/>
+    <mergeCell ref="C56:F56"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="D21:F21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>